<commit_message>
lot6f - ecart_unitaire (DETAIL) + ecart_unitaire_moyen (RESUME_LOGEMENT)
</commit_message>
<xml_diff>
--- a/02_TRAVAIL/Lot6f_CoutComplet_Menages/MASTER_CALC_CoutComplet_Menages.xlsx
+++ b/02_TRAVAIL/Lot6f_CoutComplet_Menages/MASTER_CALC_CoutComplet_Menages.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W17"/>
+  <dimension ref="A1:X17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,20 +529,25 @@
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
+          <t>ecart_unitaire</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>statut_ecart</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>statut_controle</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>code_controle</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>commentaire</t>
         </is>
@@ -622,18 +627,21 @@
       <c r="S2" t="n">
         <v>0</v>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="inlineStr">
         <is>
           <t>EQUILIBRE</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -709,18 +717,21 @@
       <c r="S3" t="n">
         <v>0</v>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="inlineStr">
         <is>
           <t>EQUILIBRE</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -796,18 +807,21 @@
       <c r="S4" t="n">
         <v>0</v>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="inlineStr">
         <is>
           <t>EQUILIBRE</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -883,18 +897,21 @@
       <c r="S5" t="n">
         <v>0</v>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" t="inlineStr">
         <is>
           <t>EQUILIBRE</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -970,18 +987,21 @@
       <c r="S6" t="n">
         <v>0</v>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="T6" t="n">
+        <v>0</v>
+      </c>
+      <c r="U6" t="inlineStr">
         <is>
           <t>EQUILIBRE</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1057,18 +1077,21 @@
       <c r="S7" t="n">
         <v>0</v>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="T7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" t="inlineStr">
         <is>
           <t>EQUILIBRE</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr"/>
       <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1144,18 +1167,21 @@
       <c r="S8" t="n">
         <v>0</v>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" t="inlineStr">
         <is>
           <t>EQUILIBRE</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
+      <c r="X8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1231,18 +1257,21 @@
       <c r="S9" t="n">
         <v>0</v>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="T9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" t="inlineStr">
         <is>
           <t>EQUILIBRE</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr"/>
       <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1318,18 +1347,21 @@
       <c r="S10" t="n">
         <v>24</v>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="T10" t="n">
+        <v>4</v>
+      </c>
+      <c r="U10" t="inlineStr">
         <is>
           <t>GAIN</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr"/>
       <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1405,18 +1437,21 @@
       <c r="S11" t="n">
         <v>30</v>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="T11" t="n">
+        <v>3</v>
+      </c>
+      <c r="U11" t="inlineStr">
         <is>
           <t>GAIN</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="V11" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
+      <c r="X11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1492,18 +1527,21 @@
       <c r="S12" t="n">
         <v>-3</v>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="T12" t="n">
+        <v>-3</v>
+      </c>
+      <c r="U12" t="inlineStr">
         <is>
           <t>PERTE</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1579,18 +1617,21 @@
       <c r="S13" t="n">
         <v>-39.48</v>
       </c>
-      <c r="T13" t="inlineStr">
+      <c r="T13" t="n">
+        <v>-9.869999999999999</v>
+      </c>
+      <c r="U13" t="inlineStr">
         <is>
           <t>PERTE</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="V13" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1666,18 +1707,21 @@
       <c r="S14" t="n">
         <v>-151.33</v>
       </c>
-      <c r="T14" t="inlineStr">
+      <c r="T14" t="n">
+        <v>-16.81</v>
+      </c>
+      <c r="U14" t="inlineStr">
         <is>
           <t>PERTE</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="V14" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1753,18 +1797,21 @@
       <c r="S15" t="n">
         <v>-81.84999999999999</v>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="T15" t="n">
+        <v>-16.37</v>
+      </c>
+      <c r="U15" t="inlineStr">
         <is>
           <t>PERTE</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="V15" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1840,18 +1887,21 @@
       <c r="S16" t="n">
         <v>-33.33</v>
       </c>
-      <c r="T16" t="inlineStr">
+      <c r="T16" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="U16" t="inlineStr">
         <is>
           <t>PERTE</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="V16" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
+      <c r="X16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1927,18 +1977,21 @@
       <c r="S17" t="n">
         <v>42</v>
       </c>
-      <c r="T17" t="inlineStr">
+      <c r="T17" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="U17" t="inlineStr">
         <is>
           <t>GAIN</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="V17" t="inlineStr">
         <is>
           <t>VALIDE</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2443,7 +2496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2482,6 +2535,11 @@
           <t>ecart_total</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ecart_unitaire_moyen</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2511,6 +2569,9 @@
       <c r="G2" t="n">
         <v>-151.33</v>
       </c>
+      <c r="H2" t="n">
+        <v>-16.81</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2540,6 +2601,9 @@
       <c r="G3" t="n">
         <v>24</v>
       </c>
+      <c r="H3" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2569,6 +2633,9 @@
       <c r="G4" t="n">
         <v>-81.84999999999999</v>
       </c>
+      <c r="H4" t="n">
+        <v>-16.37</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2598,6 +2665,9 @@
       <c r="G5" t="n">
         <v>-3</v>
       </c>
+      <c r="H5" t="n">
+        <v>-0.27</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2627,6 +2697,9 @@
       <c r="G6" t="n">
         <v>0</v>
       </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2656,6 +2729,9 @@
       <c r="G7" t="n">
         <v>42</v>
       </c>
+      <c r="H7" t="n">
+        <v>8.4</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2685,6 +2761,9 @@
       <c r="G8" t="n">
         <v>0</v>
       </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2714,6 +2793,9 @@
       <c r="G9" t="n">
         <v>0</v>
       </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2743,6 +2825,9 @@
       <c r="G10" t="n">
         <v>0</v>
       </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2772,6 +2857,9 @@
       <c r="G11" t="n">
         <v>0</v>
       </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2801,6 +2889,9 @@
       <c r="G12" t="n">
         <v>30</v>
       </c>
+      <c r="H12" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2830,6 +2921,9 @@
       <c r="G13" t="n">
         <v>-33.33</v>
       </c>
+      <c r="H13" t="n">
+        <v>-3.33</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2859,6 +2953,9 @@
       <c r="G14" t="n">
         <v>-39.48</v>
       </c>
+      <c r="H14" t="n">
+        <v>-9.869999999999999</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2886,6 +2983,9 @@
         <v>110</v>
       </c>
       <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>